<commit_message>
Updates on LLM scripts + name changes of json
</commit_message>
<xml_diff>
--- a/submission_guidelines/data_scrapes/journals_overview.xlsx
+++ b/submission_guidelines/data_scrapes/journals_overview.xlsx
@@ -675,32 +675,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nature</t>
+          <t>Annals of Mathematics</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Springer Nature</t>
+          <t>Princeton University (self-published)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0028-0836</t>
+          <t>0003-486X</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1476-4687</t>
+          <t>1939-8980</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors</t>
+          <t>https://annals.math.princeton.edu/submission-guidelines</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -708,52 +708,54 @@
           <t>scraped</t>
         </is>
       </c>
-      <c r="H2" t="b">
-        <v>1</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/robots.txt</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>The generic User-agent: * group allows these author-guideline pages, but robots.txt explicitly disallows several named AI-crawler user agents (including anthropic-ai, ClaudeBot, GPTBot) site-wide. This scraper identifies as its own named bot, not as a browser or an AI-crawler UA.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>single-anonymized; double-anonymized</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature-research/editorial-policies/peer-review</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>single-anonymized is the default; We do not release referees' identities to authors or to other reviewers unless a referee voluntarily signs their comments to the authors. Some Nature-branded journals and Communications journals offer a double-anonymized peer review option. Please visit the journal website for information on the peer review options available.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Nature Portfolio journals encourage posting of preprints of primary research manuscripts on preprint servers of the authors’ choice, authors’ or institutional websites, and open communications between researchers whether on community preprint servers or preprint commenting platforms.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature-portfolio/editorial-policies/preprints-conference-proceedings</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Springer Nature supports the responsible and transparent use of artificial intelligence where it strengthens research quality, upholds editorial independence, and preserves the integrity of the scientific and scholarly record. AI is treated as a supporting technology. Scholarly judgement, accountability, and responsibility always remain human.</t>
+          <t>Authors must be human and take full responsibility for the submission's correctness and citation accuracy. AI agents cannot be named authors. If an AI tool/LLM contributed an idea, authors must describe that idea and specify its location in the paper.</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature-portfolio/editorial-policies/ai</t>
+          <t>https://annals.math.princeton.edu/submission-guidelines</t>
         </is>
       </c>
       <c r="R2" t="b">
@@ -761,35 +763,35 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors/formatting-guide</t>
+          <t>https://annals.math.princeton.edu/submission-guidelines</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>TeX/LaTeX: If you have prepared your paper using TeX/LaTeX, we will need to convert this to Word after acceptance, before your paper can be typeset. All textual material of the paper (including references, tables, figure captions, online methods, etc.) should be included as a single .tex file.</t>
+          <t>Encouraged (class file 'aomart' from CTAN) but not required.</t>
         </is>
       </c>
       <c r="U2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors/formatting-guide</t>
+          <t>https://annals.math.princeton.edu/submission-guidelines</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>No general manuscript template. Nature provides a subject-specific ChemDraw template for chemical structures (http://www.nature.com/documents/nr-chemdraw-stylesheet.cds) and an annotated example of the summary paragraph (https://www.nature.com/documents/nature-summary-paragraph.pdf), but neither is a full manuscript template.</t>
+          <t>The 'aomart' LaTeX class file, available from CTAN -- optional, not mandatory.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>https://ctan.org/pkg/aomart</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>English; French; German</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -799,19 +801,23 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors/formatting-guide</t>
+          <t>https://annals.math.princeton.edu/submission-guidelines</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>Articles are original reports whose conclusions represent a substantial advance in understanding of an important problem and have immediate, far-reaching implications.</t>
-        </is>
-      </c>
-      <c r="AC2" t="n">
-        <v>2500</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>4300</v>
+          <t>Original mathematics research papers -- the journal documents only one general submission format.</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
@@ -820,32 +826,32 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>title; author list; acknowledgements; references</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Range reflects discipline, not a distinct article type: ~2,500 words for a 6-page article; ~4300 words for a 8-page article (physical sciences typically 6 pages, biological/clinical/social sciences typically 8).</t>
+          <t>No word/page limit stated anywhere on the page -- confirmed absence, common for pure maths journals where proof length is dictated by the mathematics, not an editorial target.</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>Titles; Text; Methods (≤3000 words); References; End notes; Life sciences and behavioural &amp; social sciences reporting guidelines; Tables; Figure legends (≤300 words); Figures; Production-quality figures; Extended Data; Supplementary Information; Chemical structures and characterization of chemical materials; Summary paragraph (≤200 words)</t>
+          <t>Abstract (~200 words or less, self-contained, no bibliography references); Bibliography</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>4-6 figures and tables combined (A 'modest' item occupies about a quarter of a page; 4 for a 6-page article, 5-6 for an 8-page article.)</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>up to 50</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>References are each numbered, ordered sequentially as they appear in the text, tables, boxes, figure legends, Methods, Extended Data tables and Extended Data figure legends. When cited in the text, reference numbers are superscript, not in brackets unless they are likely to be confused with a superscript number.</t>
+          <t>Complete references including article titles and page ranges; BibTeX preferred; DOI, Math Reviews (MathSciNet), and Zentralblatt MATH numbers included where available; arXiv number or URL for unpublished references.</t>
         </is>
       </c>
       <c r="AL2" t="inlineStr">
@@ -855,22 +861,22 @@
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>separate data and code availability statements; funding statement; author contributions; competing interest declaration</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>Word/figure/reference limits are editorial guidelines, not hard caps; final length is at the editor's discretion.</t>
+          <t>Submitted as a PDF via MSP's EditFlow system (ef.msp.org/submit/annals) -- same submission platform as Geometry &amp; Topology and Duke Mathematical Journal. LaTeX encouraged (class file 'aomart', available from CTAN) but not required. Figures must be vector graphics (EPS or PDF preferred), bundled into a single archive.</t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>Scope limited to research-submission types (excludes staff-written content: News, Careers, Obituaries, Books &amp; Arts, Futures, News &amp; Views, Technology Features, Outlooks, Comment and World View). Peer review model, preprint policy, and AI-use policy sourced from https://www.nature.com/nature-research/editorial-policies/peer-review, https://www.nature.com/nature-portfolio/editorial-policies/preprints-conference-proceedings, and https://www.nature.com/nature-portfolio/editorial-policies/ai respectively.</t>
+          <t>No article processing charges (out of scope for this schema, noted here since it was explicitly stated on the page). Non-English submissions require an English abstract in addition to the original-language one.</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>article_types[Registered Reports].total_word_limit; article_types[Registered Reports].figure_limits; article_types[Registered Reports].reference_limit</t>
+          <t>peer_review_model; preprint_policy; robots_txt_allowed</t>
         </is>
       </c>
     </row>
@@ -996,26 +1002,24 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>Correspondence</t>
+          <t>Article</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors/other-subs</t>
+          <t>https://www.nature.com/nature/for-authors/formatting-guide</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>Brief comments on topical Nature content (Editorials, World View, News, News Features, Books &amp; Arts reviews, Comment pieces or Correspondence) -- not technical comments on peer-reviewed research papers (those go to Matters Arising instead).</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>Articles are original reports whose conclusions represent a substantial advance in understanding of an important problem and have immediate, far-reaching implications.</t>
+        </is>
+      </c>
+      <c r="AC3" t="n">
+        <v>2500</v>
       </c>
       <c r="AD3" t="n">
-        <v>200</v>
+        <v>4300</v>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
@@ -1024,47 +1028,47 @@
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>title; author list; acknowledgements; references</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Hard ceiling, not a target.</t>
+          <t>Range reflects discipline, not a distinct article type: ~2,500 words for a 6-page article; ~4300 words for a 8-page article (physical sciences typically 6 pages, biological/clinical/social sciences typically 8).</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Titles; Text; Methods (≤3000 words); References; End notes; Life sciences and behavioural &amp; social sciences reporting guidelines; Tables; Figure legends (≤300 words); Figures; Production-quality figures; Extended Data; Supplementary Information; Chemical structures and characterization of chemical materials; Summary paragraph (≤200 words)</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>4-6 figures and tables combined (A 'modest' item occupies about a quarter of a page; 4 for a 6-page article, 5-6 for an 8-page article.)</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>up to 2</t>
+          <t>up to 50</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>With links to citations; further citations allowed for fact-checking only.</t>
+          <t>References are each numbered, ordered sequentially as they appear in the text, tables, boxes, figure legends, Methods, Extended Data tables and Extended Data figure legends. When cited in the text, reference numbers are superscript, not in brackets unless they are likely to be confused with a superscript number.</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>up to 4 (Collective/consortium authorship not permitted.)</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>separate data and code availability statements; funding statement; author contributions; competing interest declaration</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>Supplementary material is not permitted.</t>
+          <t>Word/figure/reference limits are editorial guidelines, not hard caps; final length is at the editor's discretion.</t>
         </is>
       </c>
       <c r="AO3" t="inlineStr">
@@ -1200,17 +1204,17 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>Matters Arising</t>
+          <t>Correspondence</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors/matters-arising</t>
+          <t>https://www.nature.com/nature/for-authors/other-subs</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>Post-publication technical comments on a Nature research paper published within the past 18 months, plus the author's Reply.</t>
+          <t>Brief comments on topical Nature content (Editorials, World View, News, News Features, Books &amp; Arts reviews, Comment pieces or Correspondence) -- not technical comments on peer-reviewed research papers (those go to Matters Arising instead).</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -1219,7 +1223,7 @@
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>1200</v>
+        <v>200</v>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
@@ -1228,47 +1232,47 @@
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>methods (may be moved to Supplementary Information)</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Target, not a hard cap ('ideally').</t>
+          <t>Hard ceiling, not a target.</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>Summary paragraph (used as the abstract); Main text; Methods (may be moved to Supplementary Information)</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>figures and tables combined (Ideally only one or two small figures or tables (stated as words, not a fixed digit, on the source page); complex ones may go into Extended Data instead (ideally no more than three such items).)</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>up to 15</t>
+          <t>up to 2</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>Same reference style as Articles.</t>
+          <t>With links to citations; further citations allowed for fact-checking only.</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>up to 4 (Collective/consortium authorship not permitted.)</t>
         </is>
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>Competing interests statement</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Supplementary material is not permitted.</t>
         </is>
       </c>
       <c r="AO4" t="inlineStr">
@@ -1404,17 +1408,17 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Matters Arising</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors/other-subs</t>
+          <t>https://www.nature.com/nature/for-authors/matters-arising</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>Focuses on one topical aspect of a field; should not focus on the author's own work.</t>
+          <t>Post-publication technical comments on a Nature research paper published within the past 18 months, plus the author's Reply.</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1422,10 +1426,8 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="AD5" t="n">
+        <v>1200</v>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
@@ -1434,32 +1436,32 @@
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>methods (may be moved to Supplementary Information)</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>No fixed word/figure/reference limit is published -- length is agreed with the commissioning editor once the synopsis is accepted. This is a confirmed 'no published number', not a gap in scraping.</t>
+          <t>Target, not a hard cap ('ideally').</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Synopsis (basic structure, material to be covered, proposed depth/arrangement)</t>
+          <t>Summary paragraph (used as the abstract); Main text; Methods (may be moved to Supplementary Information)</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>figures and tables combined (Ideally only one or two small figures or tables (stated as words, not a fixed digit, on the source page); complex ones may go into Extended Data instead (ideally no more than three such items).)</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>up to 15</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Same reference style as Articles.</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
@@ -1469,12 +1471,12 @@
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Competing interests statement</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>Most articles are commissioned, but authors wishing to submit an unsolicited Review or Perspective must do so through the online submission system via a synopsis.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AO5" t="inlineStr">
@@ -1610,7 +1612,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>Perspective</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -1620,7 +1622,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>Follows the same formatting guidelines as Reviews; more forward-looking/speculative and may be opinionated but balanced.</t>
+          <t>Focuses on one topical aspect of a field; should not focus on the author's own work.</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
@@ -1816,7 +1818,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Perspective</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -1826,7 +1828,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>Peer-reviewed; presents a new analysis of existing data rather than original data. Published only occasionally.</t>
+          <t>Follows the same formatting guidelines as Reviews; more forward-looking/speculative and may be opinionated but balanced.</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1851,12 +1853,12 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>No fixed word limit published.</t>
+          <t>No fixed word/figure/reference limit is published -- length is agreed with the commissioning editor once the synopsis is accepted. This is a confirmed 'no published number', not a gap in scraping.</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Synopsis (basic structure, material to be covered, proposed depth/arrangement)</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
@@ -1886,7 +1888,7 @@
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>Submitted via synopsis through the online submission system, with 'Analysis:' inserted before the title.</t>
+          <t>Most articles are commissioned, but authors wishing to submit an unsolicited Review or Perspective must do so through the online submission system via a synopsis.</t>
         </is>
       </c>
       <c r="AO7" t="inlineStr">
@@ -2022,17 +2024,17 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>Registered Reports</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>https://www.nature.com/nature/for-authors/registered-reports</t>
+          <t>https://www.nature.com/nature/for-authors/other-subs</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>Two-stage process: Stage 1 protocol (introduction, hypotheses, methods, analysis plan) is peer reviewed and can earn in-principle acceptance before data collection; Stage 2 is the full manuscript with results and discussion added.</t>
+          <t>Peer-reviewed; presents a new analysis of existing data rather than original data. Published only occasionally.</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
@@ -2047,7 +2049,7 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>words</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -2057,12 +2059,12 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>No fixed word limit published.</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>Stage 1: Registered Report Protocol; Stage 2: Full manuscript</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
@@ -2092,7 +2094,7 @@
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>The guidelines page doesn't state distinct word/figure/reference limits -- Stage 2 manuscripts likely follow the standard Article formatting guide, but that's not confirmed on this page.</t>
+          <t>Submitted via synopsis through the online submission system, with 'Analysis:' inserted before the title.</t>
         </is>
       </c>
       <c r="AO8" t="inlineStr">
@@ -2109,32 +2111,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The BMJ</t>
+          <t>Nature</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BMJ Publishing Group</t>
+          <t>Springer Nature</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0959-8138</t>
+          <t>0028-0836</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1756-1833</t>
+          <t>1476-4687</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://www.bmj.com/about-bmj/resources-authors</t>
+          <t>https://www.nature.com/nature/for-authors</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2142,84 +2144,78 @@
           <t>scraped</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="H9" t="b">
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>https://www.nature.com/robots.txt</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>The generic User-agent: * group allows these author-guideline pages, but robots.txt explicitly disallows several named AI-crawler user agents (including anthropic-ai, ClaudeBot, GPTBot) site-wide. This scraper identifies as its own named bot, not as a browser or an AI-crawler UA.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>single-anonymized; double-anonymized</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>https://www.nature.com/nature-research/editorial-policies/peer-review</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>single-anonymized is the default; We do not release referees' identities to authors or to other reviewers unless a referee voluntarily signs their comments to the authors. Some Nature-branded journals and Communications journals offer a double-anonymized peer review option. Please visit the journal website for information on the peer review options available.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Nature Portfolio journals encourage posting of preprints of primary research manuscripts on preprint servers of the authors’ choice, authors’ or institutional websites, and open communications between researchers whether on community preprint servers or preprint commenting platforms.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>https://www.nature.com/nature-portfolio/editorial-policies/preprints-conference-proceedings</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Springer Nature supports the responsible and transparent use of artificial intelligence where it strengthens research quality, upholds editorial independence, and preserves the integrity of the scientific and scholarly record. AI is treated as a supporting technology. Scholarly judgement, accountability, and responsibility always remain human.</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>https://www.nature.com/nature-portfolio/editorial-policies/ai</t>
+        </is>
+      </c>
+      <c r="R9" t="b">
+        <v>1</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>https://www.nature.com/nature/for-authors/formatting-guide</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>TeX/LaTeX: If you have prepared your paper using TeX/LaTeX, we will need to convert this to Word after acceptance, before your paper can be typeset. All textual material of the paper (including references, tables, figure captions, online methods, etc.) should be included as a single .tex file.</t>
+        </is>
+      </c>
+      <c r="U9" t="b">
+        <v>0</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>https://www.nature.com/nature/for-authors/formatting-guide</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>No general manuscript template. Nature provides a subject-specific ChemDraw template for chemical structures (http://www.nature.com/documents/nr-chemdraw-stylesheet.cds) and an annotated example of the summary paragraph (https://www.nature.com/documents/nature-summary-paragraph.pdf), but neither is a full manuscript template.</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -2229,22 +2225,22 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>English</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Registered Reports</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>https://www.bmj.com/about-bmj/resources-authors/article-types</t>
+          <t>https://www.nature.com/nature/for-authors/registered-reports</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>Original research articles, following IMRaD style (introduction, methods, results, discussion).</t>
+          <t>Two-stage process: Stage 1 protocol (introduction, hypotheses, methods, analysis plan) is peer reviewed and can earn in-principle acceptance before data collection; Stage 2 is the full manuscript with results and discussion added.</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -2259,7 +2255,7 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>words</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -2269,12 +2265,12 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>No fixed word count limit -- authors state their own word count at submission (main text, excluding abstract/references/tables/boxes/figures). This is a confirmed 'no published number', not a gap.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Structured abstract (≤300 words); Introduction (max 3 paragraphs); Methods; Results; Discussion</t>
+          <t>Stage 1: Registered Report Protocol; Stage 2: Full manuscript</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
@@ -2299,22 +2295,22 @@
       </c>
       <c r="AM9" t="inlineStr">
         <is>
-          <t>Title page and authorship (ICMJE criteria); Competing interests declaration; Ethics approval statement; Transparency declaration; Data sharing statement; Mandatory patient and public involvement statement; Statistical methods statement</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AN9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>The guidelines page doesn't state distinct word/figure/reference limits -- Stage 2 manuscripts likely follow the standard Article formatting guide, but that's not confirmed on this page.</t>
         </is>
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>Scope limited to research-submission types -- excludes BMJ Careers (pure pitch, no format), Obituaries (family submissions), and 'Summary of NICE Guidelines' (solely commissioned, no author-submission path). Peer review model, preprint policy, and AI-use policy pages have not been fetched yet (separate task from this extraction pass).</t>
+          <t>Scope limited to research-submission types (excludes staff-written content: News, Careers, Obituaries, Books &amp; Arts, Futures, News &amp; Views, Technology Features, Outlooks, Comment and World View). Peer review model, preprint policy, and AI-use policy sourced from https://www.nature.com/nature-research/editorial-policies/peer-review, https://www.nature.com/nature-portfolio/editorial-policies/preprints-conference-proceedings, and https://www.nature.com/nature-portfolio/editorial-policies/ai respectively.</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>article_types[State of the Art Reviews].total_word_limit; peer_review_model; preprint_policy; ai_use_policy; latex_accepted; template_provided; languages_accepted</t>
+          <t>article_types[Registered Reports].total_word_limit; article_types[Registered Reports].figure_limits; article_types[Registered Reports].reference_limit</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2442,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>Research Methods and Reporting (RMR)</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -2456,7 +2452,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>Articles on research methodology and reporting standards.</t>
+          <t>Original research articles, following IMRaD style (introduction, methods, results, discussion).</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
@@ -2481,12 +2477,12 @@
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>No fixed word count limit -- same 'make every word count' guidance as Research.</t>
+          <t>No fixed word count limit -- authors state their own word count at submission (main text, excluding abstract/references/tables/boxes/figures). This is a confirmed 'no published number', not a gap.</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>Title and standfirst (100-150 words); Introduction; Text (subheaded)</t>
+          <t>Structured abstract (≤300 words); Introduction (max 3 paragraphs); Methods; Results; Discussion</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
@@ -2511,7 +2507,7 @@
       </c>
       <c r="AM10" t="inlineStr">
         <is>
-          <t>Title page and authorship (ICMJE criteria); Competing interests declaration; Ethics approval statement; Transparency declaration</t>
+          <t>Title page and authorship (ICMJE criteria); Competing interests declaration; Ethics approval statement; Transparency declaration; Data sharing statement; Mandatory patient and public involvement statement; Statistical methods statement</t>
         </is>
       </c>
       <c r="AN10" t="inlineStr">
@@ -2658,7 +2654,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Research Methods and Reporting (RMR)</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
@@ -2668,14 +2664,18 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>International-readership pieces for policy makers, health professionals, and doctors of all disciplines; avoids jargon.</t>
-        </is>
-      </c>
-      <c r="AC11" t="n">
-        <v>2000</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>2000</v>
+          <t>Articles on research methodology and reporting standards.</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
@@ -2689,12 +2689,12 @@
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>No fixed word count limit -- same 'make every word count' guidance as Research.</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Title and standfirst (100-150 words); Introduction; Text (subheaded)</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
@@ -2704,7 +2704,7 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>up to 20</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="AN11" t="inlineStr">
         <is>
-          <t>Up to 3 non-text items (box, figure, or table).</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AO11" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>Editorials</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
@@ -2876,16 +2876,14 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>Scholarly, balanced, evidence-based responses to something topical; usually 1-3 authors, max 4 (5 if the extra author is a patient).</t>
-        </is>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>International-readership pieces for policy makers, health professionals, and doctors of all disciplines; avoids jargon.</t>
+        </is>
+      </c>
+      <c r="AC12" t="n">
+        <v>2000</v>
       </c>
       <c r="AD12" t="n">
-        <v>800</v>
+        <v>2000</v>
       </c>
       <c r="AE12" t="inlineStr">
         <is>
@@ -2899,7 +2897,7 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>'Up to 800 words' -- explicit ceiling.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
@@ -2914,7 +2912,7 @@
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>12-20</t>
+          <t>up to 20</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
@@ -2924,17 +2922,17 @@
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>up to 4 (5 allowed only if the extra author is a patient.)</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Title page and authorship (ICMJE criteria); Competing interests declaration; Ethics approval statement; Transparency declaration</t>
         </is>
       </c>
       <c r="AN12" t="inlineStr">
         <is>
-          <t>Invited only. Authors must be free of relevant financial ties to industry (since 2014 policy).</t>
+          <t>Up to 3 non-text items (box, figure, or table).</t>
         </is>
       </c>
       <c r="AO12" t="inlineStr">
@@ -3076,7 +3074,7 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>Personal Views</t>
+          <t>Editorials</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
@@ -3086,14 +3084,16 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>A strong, novel, well-argued personal viewpoint. Published online first on BMJ Opinion; may not appear in print.</t>
-        </is>
-      </c>
-      <c r="AC13" t="n">
-        <v>600</v>
+          <t>Scholarly, balanced, evidence-based responses to something topical; usually 1-3 authors, max 4 (5 if the extra author is a patient).</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="AD13" t="n">
-        <v>600</v>
+        <v>800</v>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
@@ -3107,7 +3107,7 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>'Up to 800 words' -- explicit ceiling.</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
@@ -3122,7 +3122,7 @@
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>up to 10</t>
+          <t>12-20</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>up to 4 (5 allowed only if the extra author is a patient.)</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Invited only. Authors must be free of relevant financial ties to industry (since 2014 policy).</t>
         </is>
       </c>
       <c r="AO13" t="inlineStr">
@@ -3284,7 +3284,7 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>BMJ Opinion</t>
+          <t>Personal Views</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
@@ -3294,14 +3294,14 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>Comment and opinion from BMJ's international community of readers, authors, and editors, on medicine/healthcare/publishing.</t>
+          <t>A strong, novel, well-argued personal viewpoint. Published online first on BMJ Opinion; may not appear in print.</t>
         </is>
       </c>
       <c r="AC14" t="n">
-        <v>650</v>
+        <v>600</v>
       </c>
       <c r="AD14" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
@@ -3330,7 +3330,7 @@
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>up to 10</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="AN14" t="inlineStr">
         <is>
-          <t>Submitted via email (blogs@bmj.com), not the main submission system.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AO14" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>Rapid responses</t>
+          <t>BMJ Opinion</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr">
@@ -3502,18 +3502,14 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>Electronic letters to the editor -- the only route for a letter to appear in print/bmj.com; all print letters originate as rapid responses.</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+          <t>Comment and opinion from BMJ's international community of readers, authors, and editors, on medicine/healthcare/publishing.</t>
+        </is>
+      </c>
+      <c r="AC15" t="n">
+        <v>650</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>800</v>
       </c>
       <c r="AE15" t="inlineStr">
         <is>
@@ -3527,7 +3523,7 @@
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>No word limit stated (n/a in the source table).</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AH15" t="inlineStr">
@@ -3562,7 +3558,7 @@
       </c>
       <c r="AN15" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Submitted via email (blogs@bmj.com), not the main submission system.</t>
         </is>
       </c>
       <c r="AO15" t="inlineStr">
@@ -3704,7 +3700,7 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>Clinical Updates</t>
+          <t>Rapid responses</t>
         </is>
       </c>
       <c r="AA16" t="inlineStr">
@@ -3714,14 +3710,18 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>Up-to-date overview of a clinical condition, evidence-based, aimed at non-specialists.</t>
-        </is>
-      </c>
-      <c r="AC16" t="n">
-        <v>1800</v>
-      </c>
-      <c r="AD16" t="n">
-        <v>1800</v>
+          <t>Electronic letters to the editor -- the only route for a letter to appear in print/bmj.com; all print letters originate as rapid responses.</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>No word limit stated (n/a in the source table).</t>
         </is>
       </c>
       <c r="AH16" t="inlineStr">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>up to 40</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AK16" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>Practice Pointer</t>
+          <t>Clinical Updates</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
@@ -3922,14 +3922,14 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Up-to-date overview of a clinical condition, evidence-based, aimed at non-specialists.</t>
         </is>
       </c>
       <c r="AC17" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="AD17" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="AE17" t="inlineStr">
         <is>
@@ -3958,7 +3958,7 @@
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>up to 20</t>
+          <t>up to 40</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>Easily Missed</t>
+          <t>Practice Pointer</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>10 Minute Consultation</t>
+          <t>Easily Missed</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
@@ -4342,10 +4342,10 @@
         </is>
       </c>
       <c r="AC19" t="n">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="AD19" t="n">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="AE19" t="inlineStr">
         <is>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>up to 10</t>
+          <t>up to 20</t>
         </is>
       </c>
       <c r="AK19" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>Sustainable Practice</t>
+          <t>10 Minute Consultation</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
@@ -4550,10 +4550,10 @@
         </is>
       </c>
       <c r="AC20" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="AD20" t="n">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
@@ -4582,7 +4582,7 @@
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>up to 10</t>
         </is>
       </c>
       <c r="AK20" t="inlineStr">
@@ -4744,7 +4744,7 @@
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>What Your Patient Is Thinking (WYPIT)</t>
+          <t>Sustainable Practice</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
@@ -4758,10 +4758,10 @@
         </is>
       </c>
       <c r="AC21" t="n">
-        <v>650</v>
+        <v>400</v>
       </c>
       <c r="AD21" t="n">
-        <v>650</v>
+        <v>700</v>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
@@ -4775,7 +4775,7 @@
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>Includes the closing 'What You Need To Know' summary box.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AH21" t="inlineStr">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>Minerva Pictures</t>
+          <t>What Your Patient Is Thinking (WYPIT)</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
@@ -4966,10 +4966,10 @@
         </is>
       </c>
       <c r="AC22" t="n">
-        <v>150</v>
+        <v>650</v>
       </c>
       <c r="AD22" t="n">
-        <v>150</v>
+        <v>650</v>
       </c>
       <c r="AE22" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Includes the closing 'What You Need To Know' summary box.</t>
         </is>
       </c>
       <c r="AH22" t="inlineStr">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>Endgames</t>
+          <t>Minerva Pictures</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
@@ -5173,19 +5173,15 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="AC23" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AD23" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
+      <c r="AC23" t="n">
+        <v>150</v>
+      </c>
+      <c r="AD23" t="n">
+        <v>150</v>
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>words</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -5230,7 +5226,7 @@
       </c>
       <c r="AN23" t="inlineStr">
         <is>
-          <t>150-word vignette (case history) section plus a 200-word answer section -- two separately limited parts of one piece, not a single total word count. See template referenced on the source page.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AO23" t="inlineStr">
@@ -5372,7 +5368,7 @@
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>State of the Art Reviews</t>
+          <t>Endgames</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
@@ -5442,7 +5438,7 @@
       </c>
       <c r="AN24" t="inlineStr">
         <is>
-          <t>Word limit cell was blank in the source table -- genuinely not checked, not a confirmed absence.</t>
+          <t>150-word vignette (case history) section plus a 200-word answer section -- two separately limited parts of one piece, not a single total word count. See template referenced on the source page.</t>
         </is>
       </c>
       <c r="AO24" t="inlineStr">
@@ -5459,27 +5455,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Annals of Mathematics</t>
+          <t>The BMJ</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Princeton University (self-published)</t>
+          <t>BMJ Publishing Group</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0003-486X</t>
+          <t>0959-8138</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1939-8980</t>
+          <t>1756-1833</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://annals.math.princeton.edu/submission-guidelines</t>
+          <t>https://www.bmj.com/about-bmj/resources-authors</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -5534,63 +5530,67 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Authors must be human and take full responsibility for the submission's correctness and citation accuracy. AI agents cannot be named authors. If an AI tool/LLM contributed an idea, authors must describe that idea and specify its location in the paper.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>https://annals.math.princeton.edu/submission-guidelines</t>
-        </is>
-      </c>
-      <c r="R25" t="b">
-        <v>1</v>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>https://annals.math.princeton.edu/submission-guidelines</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>Encouraged (class file 'aomart' from CTAN) but not required.</t>
-        </is>
-      </c>
-      <c r="U25" t="b">
-        <v>1</v>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>https://annals.math.princeton.edu/submission-guidelines</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>The 'aomart' LaTeX class file, available from CTAN -- optional, not mandatory.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>https://ctan.org/pkg/aomart</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>English; French; German</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>Article</t>
+          <t>State of the Art Reviews</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>https://annals.math.princeton.edu/submission-guidelines</t>
+          <t>https://www.bmj.com/about-bmj/resources-authors/article-types</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>Original mathematics research papers -- the journal documents only one general submission format.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>words</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
@@ -5615,12 +5615,12 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>No word/page limit stated anywhere on the page -- confirmed absence, common for pure maths journals where proof length is dictated by the mathematics, not an editorial target.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>Abstract (~200 words or less, self-contained, no bibliography references); Bibliography</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="AK25" t="inlineStr">
         <is>
-          <t>Complete references including article titles and page ranges; BibTeX preferred; DOI, Math Reviews (MathSciNet), and Zentralblatt MATH numbers included where available; arXiv number or URL for unpublished references.</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="AL25" t="inlineStr">
@@ -5650,17 +5650,17 @@
       </c>
       <c r="AN25" t="inlineStr">
         <is>
-          <t>Submitted as a PDF via MSP's EditFlow system (ef.msp.org/submit/annals) -- same submission platform as Geometry &amp; Topology and Duke Mathematical Journal. LaTeX encouraged (class file 'aomart', available from CTAN) but not required. Figures must be vector graphics (EPS or PDF preferred), bundled into a single archive.</t>
+          <t>Word limit cell was blank in the source table -- genuinely not checked, not a confirmed absence.</t>
         </is>
       </c>
       <c r="AO25" t="inlineStr">
         <is>
-          <t>No article processing charges (out of scope for this schema, noted here since it was explicitly stated on the page). Non-English submissions require an English abstract in addition to the original-language one.</t>
+          <t>Scope limited to research-submission types -- excludes BMJ Careers (pure pitch, no format), Obituaries (family submissions), and 'Summary of NICE Guidelines' (solely commissioned, no author-submission path). Peer review model, preprint policy, and AI-use policy pages have not been fetched yet (separate task from this extraction pass).</t>
         </is>
       </c>
       <c r="AP25" t="inlineStr">
         <is>
-          <t>peer_review_model; preprint_policy; robots_txt_allowed</t>
+          <t>article_types[State of the Art Reviews].total_word_limit; peer_review_model; preprint_policy; ai_use_policy; latex_accepted; template_provided; languages_accepted</t>
         </is>
       </c>
     </row>

</xml_diff>